<commit_message>
Rename the Producer AI area to Model development and release
The area is the job of owning a model (purpose and design, evaluation
before use, the base model, release to others), not the producer role,
so its id becomes model_development in the sheet, ai_areas.json,
mapping_rules.json and scope_rules.json. The role and the producer bank
keep their names. TODO: all open decisions settled; the next session
starts with the mapping pilot.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LfWLLRUPBVgScvEVMJMnXw
</commit_message>
<xml_diff>
--- a/data/ai/authoring/ai_areas.xlsx
+++ b/data/ai/authoring/ai_areas.xlsx
@@ -632,12 +632,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>producer</t>
+          <t>model_development</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Producer</t>
+          <t>Model development and release</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Rename the model_development AI area to Model building
Same pattern as the other usage areas (Code generation, Vendor AI) and
the intake wording 'Do you build AI', and no longer reads like a second
Model component. Id model_building in the sheet, ai_areas.json,
mapping_rules.json, scope_rules.json, tests and docs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LfWLLRUPBVgScvEVMJMnXw
</commit_message>
<xml_diff>
--- a/data/ai/authoring/ai_areas.xlsx
+++ b/data/ai/authoring/ai_areas.xlsx
@@ -632,12 +632,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>model_development</t>
+          <t>model_building</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Model development and release</t>
+          <t>Model building</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
After the pilot re-run: model is IP, people impact, 4 more foundation, other_areas
- Model impact back to assets; new impact people on customer_facing and output
- MAP 3.4, MEASURE 1.2, MEASURE 3.1, MANAGE 1.4 foundation (12 in all)
- Mapping input carries other_areas (id, name, applies_to, covers from the AI areas
  sheet); drafter leaves out, evaluator fails, rows belonging to another area or with a
  why that would read the same for any area
- Pilot re-run deleted (mapping.json, mapping.xlsx, inputs); audit trail kept
- TODO: next pilot on model and agent with expectations

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LfWLLRUPBVgScvEVMJMnXw
</commit_message>
<xml_diff>
--- a/data/ai/authoring/ai_areas.xlsx
+++ b/data/ai/authoring/ai_areas.xlsx
@@ -578,7 +578,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>process, data</t>
+          <t>process, data, people</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>process</t>
+          <t>process, people</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>assets, process</t>
+          <t>assets</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Batch 1 review: model building narrowed to the activity, bias and TEVV at Output
Model building covers: build or tune, base models, release, limits told, withdraw;
testing answers is Output, weights are Model, data is Test, tuning and evaluation data.
Output covers add biased answers and TEVV for everyone. internal_process gets no people
impact. All recorded areas are stale by the sheet change; TODO lists the batches.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LfWLLRUPBVgScvEVMJMnXw
</commit_message>
<xml_diff>
--- a/data/ai/authoring/ai_areas.xlsx
+++ b/data/ai/authoring/ai_areas.xlsx
@@ -657,7 +657,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>The org owns a model: built from scratch, or modified by domain-specific training or tuning of an existing model. If the model is given to others (API, weights, embedded in a product), recipients depend on it: limits not communicated, unsafe changes, no way to withdraw a release.</t>
+          <t>The org builds or tunes its own model: from scratch, or by domain-specific training or tuning of an existing model. The activity: the base models and components chosen, how building and tuning are run and changed, releasing versions to others (API, weights, embedded in a product), telling recipients the limits, and withdrawing a release. Not here: testing how accurate, consistent or fair its answers are (Output), the weights and versions as IP (Model), the training and test data (Test, tuning and evaluation data).</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Answers that are wrong and are then trusted by people and systems, so they become a wrong decision or action. Two kinds: steered by an attacker (prompt injection through user input or retrieved content, poisoned answers), or simply inaccurate with no attacker (made-up facts, different answers to the same question, quality drifting over time).</t>
+          <t>Answers that are wrong and are then trusted by people and systems, so they become a wrong decision or action. Two kinds: steered by an attacker (prompt injection through user input or retrieved content, poisoned answers), or simply poor with no attacker (made-up facts, different answers to the same question, quality drifting over time, or biased: treating people or groups unequally). Testing answers for accuracy, consistency and bias (TEVV) is done here for everyone, including organisations that build their own model.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Areas: internal_process and customer_facing ask about catching and auditing high-impact output
Wrong or biased output is tested at Output; these usage areas ask how staff or customers
check, report and challenge it, and how high-impact decisions are caught and audited.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LfWLLRUPBVgScvEVMJMnXw
</commit_message>
<xml_diff>
--- a/data/ai/authoring/ai_areas.xlsx
+++ b/data/ai/authoring/ai_areas.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>AI output driving internal decisions and workflows (HR, finance, approvals, operations). Staff are the users: over-reliance, misuse by insiders, decisions made on wrong output.</t>
+          <t>AI output driving internal decisions and workflows (HR, finance, approvals, operations). Staff are the users: over-reliance, misuse by insiders, decisions made on wrong output. Whether the output is wrong or biased is tested at Output; here: how staff check, challenge and override it, and how high-impact decisions made on it are caught and audited.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Public users can attack the AI (prompt injection, abuse), and AI output reaches customers directly: wrong, harmful or leaked answers in front of customers.</t>
+          <t>Public users can attack the AI (prompt injection, abuse), and AI output reaches customers directly: wrong, harmful or leaked answers in front of customers. Whether answers are wrong or biased is tested at Output; here: how customers report problems and negative feedback, and how high-impact answers are caught and audited.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">

</xml_diff>